<commit_message>
First round of testing done, M1 M2 and partial M8. Develope ddata analysis tools.
</commit_message>
<xml_diff>
--- a/docs/Energy_Test_Results.xlsx
+++ b/docs/Energy_Test_Results.xlsx
@@ -8,24 +8,37 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://memsystech-my.sharepoint.com/personal/c_valencia_memsys_nl/Documents/Documents/Github/UniversalMotorModule/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="233" documentId="11_BF2D1F772994728708AE13DA929BFF4427475816" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA63F3F3-F1D0-4593-A3B7-A057C3BB626B}"/>
+  <xr:revisionPtr revIDLastSave="289" documentId="11_BF2D1F772994728708AE13DA929BFF4427475816" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D502468-C27B-4E29-A734-46993C13685A}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Motor 1" sheetId="1" r:id="rId1"/>
     <sheet name="Motor 2" sheetId="2" r:id="rId2"/>
-    <sheet name="Motor 11A" sheetId="6" r:id="rId3"/>
-    <sheet name="Motor 8" sheetId="3" r:id="rId4"/>
+    <sheet name="Motor 8" sheetId="3" r:id="rId3"/>
+    <sheet name="Motor 11A" sheetId="6" r:id="rId4"/>
     <sheet name="Motor 10" sheetId="5" r:id="rId5"/>
     <sheet name="Motor 11D" sheetId="7" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1291" uniqueCount="204">
   <si>
     <t>Motor 1: ____________________</t>
   </si>
@@ -543,9 +556,6 @@
     <t>Thrust (N)</t>
   </si>
   <si>
-    <t>Not doable</t>
-  </si>
-  <si>
     <t>2500 travel steps</t>
   </si>
   <si>
@@ -631,6 +641,15 @@
   </si>
   <si>
     <t>Reverse direction</t>
+  </si>
+  <si>
+    <t>Actuator Power (W)</t>
+  </si>
+  <si>
+    <t>Not doable, minimum voltage for current driver 3.8V</t>
+  </si>
+  <si>
+    <t>Actuator Energy (mJ) Normal direction-Reverse direction</t>
   </si>
 </sst>
 </file>
@@ -720,7 +739,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -738,6 +757,9 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -757,309 +779,269 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>600075</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>161925</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>29346</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>10351</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>428625</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>172276</xdr:rowOff>
     </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="10" name="Group 9">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ADC55EB0-20B1-CB1F-B0F9-A98D28A7D536}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9E2EDC84-A763-C352-FB99-ABD7E30749B4}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="8734425" y="238125"/>
-          <a:ext cx="5525271" cy="5915851"/>
+          <a:off x="11344275" y="590550"/>
+          <a:ext cx="5753100" cy="5915851"/>
+          <a:chOff x="8753475" y="228600"/>
+          <a:chExt cx="5753100" cy="5915851"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>447675</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>438150</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="4" name="Straight Arrow Connector 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{45EACF28-BBD1-4D84-C8FA-3990D2299283}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr/>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm flipV="1">
-          <a:off x="12849225" y="1571625"/>
-          <a:ext cx="1209675" cy="2790825"/>
-        </a:xfrm>
-        <a:prstGeom prst="straightConnector1">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="57150">
+      </xdr:grpSpPr>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="2" name="Picture 1">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ADC55EB0-20B1-CB1F-B0F9-A98D28A7D536}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8753475" y="228600"/>
+            <a:ext cx="5525271" cy="5915851"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+      </xdr:pic>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="4" name="Straight Arrow Connector 3">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{45EACF28-BBD1-4D84-C8FA-3990D2299283}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm flipV="1">
+            <a:off x="12849225" y="1571625"/>
+            <a:ext cx="1209675" cy="2790825"/>
+          </a:xfrm>
+          <a:prstGeom prst="straightConnector1">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="57150">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="5" name="TextBox 4">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D6A258EA-F46B-BD14-A802-A24B9A301AB9}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="13725525" y="2857500"/>
+            <a:ext cx="781050" cy="571500"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
           <a:solidFill>
-            <a:srgbClr val="FF0000"/>
+            <a:schemeClr val="lt1"/>
           </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>104775</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>276225</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="5" name="TextBox 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D6A258EA-F46B-BD14-A802-A24B9A301AB9}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="13725525" y="2771775"/>
-          <a:ext cx="781050" cy="571500"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
+          <a:ln w="9525" cmpd="sng">
+            <a:solidFill>
+              <a:schemeClr val="lt1">
+                <a:shade val="50000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100"/>
+              <a:t>Normal direction</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:endParaRPr lang="en-NL" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="6" name="Straight Arrow Connector 5">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{17462283-02E2-4DD0-9C4F-5032F0DFDEA8}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm flipH="1">
+            <a:off x="10982325" y="838200"/>
+            <a:ext cx="1181100" cy="2743200"/>
+          </a:xfrm>
+          <a:prstGeom prst="straightConnector1">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="57150">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="8" name="TextBox 7">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3EEF6FE1-53C3-4DDC-AAD5-AC479F2E1BA6}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="10306050" y="2790825"/>
+            <a:ext cx="781050" cy="571500"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
           <a:solidFill>
-            <a:schemeClr val="lt1">
-              <a:shade val="50000"/>
-            </a:schemeClr>
+            <a:schemeClr val="lt1"/>
           </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100"/>
-            <a:t>Normal direction</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-NL" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>371475</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>104775</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="6" name="Straight Arrow Connector 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{17462283-02E2-4DD0-9C4F-5032F0DFDEA8}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr/>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm flipH="1">
-          <a:off x="10982325" y="838200"/>
-          <a:ext cx="1181100" cy="2743200"/>
-        </a:xfrm>
-        <a:prstGeom prst="straightConnector1">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="57150">
-          <a:solidFill>
-            <a:srgbClr val="FF0000"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>342900</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>514350</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="8" name="TextBox 7">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3EEF6FE1-53C3-4DDC-AAD5-AC479F2E1BA6}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="10306050" y="2790825"/>
-          <a:ext cx="781050" cy="571500"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:solidFill>
-            <a:schemeClr val="lt1">
-              <a:shade val="50000"/>
-            </a:schemeClr>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100"/>
-            <a:t>Reverse direction</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100"/>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-NL" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
+          <a:ln w="9525" cmpd="sng">
+            <a:solidFill>
+              <a:schemeClr val="lt1">
+                <a:shade val="50000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100"/>
+              <a:t>Reverse direction</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:endParaRPr lang="en-US" sz="1100"/>
+          </a:p>
+          <a:p>
+            <a:endParaRPr lang="en-NL" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+    </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -1069,16 +1051,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>180975</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>457859</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>29234</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>105720</xdr:rowOff>
+      <xdr:rowOff>153345</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1101,7 +1083,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8743950" y="238125"/>
+          <a:off x="10144125" y="285750"/>
           <a:ext cx="4725059" cy="6773220"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1115,6 +1097,55 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>553038</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>134299</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{07894564-6668-5990-8F49-3BE8CDB44C95}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8743950" y="238125"/>
+          <a:ext cx="4210638" cy="6801799"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1152,55 +1183,6 @@
         <a:xfrm>
           <a:off x="8743950" y="238125"/>
           <a:ext cx="3219899" cy="3372321"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>553038</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>134299</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{07894564-6668-5990-8F49-3BE8CDB44C95}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="8743950" y="238125"/>
-          <a:ext cx="4210638" cy="6801799"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1634,7 +1616,7 @@
       <c r="F5" s="7"/>
       <c r="G5" s="7"/>
       <c r="H5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1651,7 +1633,7 @@
         <v>5</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>6</v>
+        <v>201</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>7</v>
@@ -1668,22 +1650,22 @@
         <v>10</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H7" t="s">
-        <v>172</v>
+        <v>202</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1697,7 +1679,10 @@
         <v>4</v>
       </c>
       <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
+      <c r="E8" s="3">
+        <f t="shared" ref="E8:E9" si="0">G8/F8</f>
+        <v>0.6</v>
+      </c>
       <c r="F8" s="3">
         <v>25000</v>
       </c>
@@ -1716,7 +1701,10 @@
         <v>4.5</v>
       </c>
       <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
+      <c r="E9" s="3">
+        <f t="shared" si="0"/>
+        <v>0.8</v>
+      </c>
       <c r="F9" s="3">
         <v>25000</v>
       </c>
@@ -1735,7 +1723,10 @@
         <v>5</v>
       </c>
       <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
+      <c r="E10" s="3">
+        <f>G10/F10</f>
+        <v>1.04</v>
+      </c>
       <c r="F10" s="3">
         <v>25000</v>
       </c>
@@ -1754,7 +1745,7 @@
       <c r="F12" s="7"/>
       <c r="G12" s="7"/>
       <c r="H12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1771,7 +1762,7 @@
         <v>5</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>6</v>
+        <v>201</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>7</v>
@@ -1788,19 +1779,19 @@
         <v>10</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -1814,7 +1805,10 @@
         <v>3.6</v>
       </c>
       <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
+      <c r="E15" s="3">
+        <f t="shared" ref="E15:E17" si="1">G15/F15</f>
+        <v>0.38095238095238093</v>
+      </c>
       <c r="F15" s="3">
         <v>10500</v>
       </c>
@@ -1833,7 +1827,10 @@
         <v>4.5</v>
       </c>
       <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
+      <c r="E16" s="3">
+        <f t="shared" si="1"/>
+        <v>0.63809523809523805</v>
+      </c>
       <c r="F16" s="3">
         <v>10500</v>
       </c>
@@ -1852,7 +1849,10 @@
         <v>4.5</v>
       </c>
       <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
+      <c r="E17" s="3">
+        <f t="shared" si="1"/>
+        <v>0.69523809523809521</v>
+      </c>
       <c r="F17" s="3">
         <v>10500</v>
       </c>
@@ -1871,7 +1871,7 @@
       <c r="F19" s="7"/>
       <c r="G19" s="7"/>
       <c r="H19" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -1888,7 +1888,7 @@
         <v>5</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>6</v>
+        <v>201</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>7</v>
@@ -1905,19 +1905,19 @@
         <v>10</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -1931,7 +1931,10 @@
         <v>3.9</v>
       </c>
       <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
+      <c r="E22" s="3">
+        <f t="shared" ref="E22:E24" si="2">G22/F22</f>
+        <v>0.35535714285714287</v>
+      </c>
       <c r="F22" s="3">
         <v>2800</v>
       </c>
@@ -1950,7 +1953,10 @@
         <v>5</v>
       </c>
       <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
+      <c r="E23" s="3">
+        <f t="shared" si="2"/>
+        <v>0.5535714285714286</v>
+      </c>
       <c r="F23" s="3">
         <v>2800</v>
       </c>
@@ -1969,7 +1975,10 @@
         <v>5</v>
       </c>
       <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
+      <c r="E24" s="3">
+        <f t="shared" si="2"/>
+        <v>0.6071428571428571</v>
+      </c>
       <c r="F24" s="3">
         <v>2800</v>
       </c>
@@ -1988,7 +1997,7 @@
       <c r="F26" s="7"/>
       <c r="G26" s="7"/>
       <c r="H26" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -2005,7 +2014,7 @@
         <v>5</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>6</v>
+        <v>201</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>7</v>
@@ -2022,19 +2031,19 @@
         <v>10</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -2048,7 +2057,10 @@
         <v>4.9000000000000004</v>
       </c>
       <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
+      <c r="E29" s="3">
+        <f t="shared" ref="E29:E31" si="3">G29/F29</f>
+        <v>0.53071428571428569</v>
+      </c>
       <c r="F29" s="3">
         <v>1400</v>
       </c>
@@ -2067,7 +2079,10 @@
         <v>5.5</v>
       </c>
       <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
+      <c r="E30" s="3">
+        <f t="shared" si="3"/>
+        <v>0.8571428571428571</v>
+      </c>
       <c r="F30" s="3">
         <v>1400</v>
       </c>
@@ -2086,7 +2101,10 @@
         <v>5.3</v>
       </c>
       <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
+      <c r="E31" s="3">
+        <f t="shared" si="3"/>
+        <v>0.9285714285714286</v>
+      </c>
       <c r="F31" s="3">
         <v>1400</v>
       </c>
@@ -2105,7 +2123,7 @@
       <c r="F33" s="7"/>
       <c r="G33" s="7"/>
       <c r="H33" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
@@ -2122,13 +2140,13 @@
         <v>5</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>6</v>
+        <v>201</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>8</v>
+        <v>203</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
@@ -2139,19 +2157,19 @@
         <v>10</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
@@ -2162,7 +2180,7 @@
         <v>12</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
@@ -2170,7 +2188,7 @@
         <v>1400</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
@@ -2181,7 +2199,7 @@
         <v>14</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
@@ -2189,7 +2207,7 @@
         <v>1400</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
@@ -2200,7 +2218,7 @@
         <v>16</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
@@ -2208,7 +2226,7 @@
         <v>1400</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
@@ -3121,7 +3139,7 @@
         <v>80</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D119" s="2" t="s">
         <v>82</v>
@@ -3129,7 +3147,7 @@
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B120" s="3" t="s">
         <v>83</v>
@@ -3138,12 +3156,12 @@
         <v>7.5</v>
       </c>
       <c r="D120" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B121" s="3" t="s">
         <v>83</v>
@@ -3152,7 +3170,7 @@
         <v>10</v>
       </c>
       <c r="D121" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.25">
@@ -3257,11 +3275,12 @@
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -3286,7 +3305,7 @@
       <c r="F5" s="7"/>
       <c r="G5" s="7"/>
       <c r="H5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -3336,7 +3355,10 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
+      <c r="E8" s="3">
+        <f t="shared" ref="E8:E9" si="0">G8/F8</f>
+        <v>0.41346153846153844</v>
+      </c>
       <c r="F8" s="3">
         <v>10400</v>
       </c>
@@ -3355,7 +3377,10 @@
         <v>4.5</v>
       </c>
       <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
+      <c r="E9" s="3">
+        <f t="shared" si="0"/>
+        <v>0.63461538461538458</v>
+      </c>
       <c r="F9" s="3">
         <v>10400</v>
       </c>
@@ -3374,7 +3399,10 @@
         <v>6.3</v>
       </c>
       <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
+      <c r="E10" s="3">
+        <f>G10/F10</f>
+        <v>0.86538461538461542</v>
+      </c>
       <c r="F10" s="3">
         <v>10400</v>
       </c>
@@ -3393,7 +3421,7 @@
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
       <c r="H13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -3443,7 +3471,10 @@
         <v>4.9000000000000004</v>
       </c>
       <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
+      <c r="E16" s="3">
+        <f>G16/F16</f>
+        <v>0.30263157894736842</v>
+      </c>
       <c r="F16" s="3">
         <v>760</v>
       </c>
@@ -3462,7 +3493,10 @@
         <v>5.8</v>
       </c>
       <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
+      <c r="E17" s="3">
+        <f t="shared" ref="E17:E18" si="1">G17/F17</f>
+        <v>0.46710526315789475</v>
+      </c>
       <c r="F17" s="3">
         <v>760</v>
       </c>
@@ -3481,7 +3515,10 @@
         <v>7</v>
       </c>
       <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
+      <c r="E18" s="3">
+        <f t="shared" si="1"/>
+        <v>0.61842105263157898</v>
+      </c>
       <c r="F18" s="3">
         <v>760</v>
       </c>
@@ -3491,7 +3528,7 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -3511,7 +3548,7 @@
       <c r="F22" s="7"/>
       <c r="G22" s="7"/>
       <c r="H22" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -3539,7 +3576,7 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>10</v>
@@ -3552,7 +3589,7 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>12</v>
@@ -3561,7 +3598,10 @@
         <v>3.7</v>
       </c>
       <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
+      <c r="E25" s="3">
+        <f>G25/F25</f>
+        <v>0.41346153846153844</v>
+      </c>
       <c r="F25" s="3">
         <v>10400</v>
       </c>
@@ -3571,7 +3611,7 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>14</v>
@@ -3580,7 +3620,10 @@
         <v>5.8</v>
       </c>
       <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
+      <c r="E26" s="3">
+        <f>G26/F26</f>
+        <v>0.625</v>
+      </c>
       <c r="F26" s="3">
         <v>10400</v>
       </c>
@@ -3590,7 +3633,7 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>16</v>
@@ -3599,7 +3642,10 @@
         <v>6</v>
       </c>
       <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
+      <c r="E27" s="3">
+        <f>G27/F27</f>
+        <v>0.86538461538461542</v>
+      </c>
       <c r="F27" s="3">
         <v>10400</v>
       </c>
@@ -3618,7 +3664,7 @@
       <c r="F30" s="7"/>
       <c r="G30" s="7"/>
       <c r="H30" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
@@ -3646,7 +3692,7 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>10</v>
@@ -3659,7 +3705,7 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>12</v>
@@ -3668,7 +3714,10 @@
         <v>3.9</v>
       </c>
       <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
+      <c r="E33" s="3">
+        <f>G33/F33</f>
+        <v>0.31578947368421051</v>
+      </c>
       <c r="F33" s="3">
         <v>760</v>
       </c>
@@ -3678,7 +3727,7 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>14</v>
@@ -3687,7 +3736,10 @@
         <v>6</v>
       </c>
       <c r="D34" s="3"/>
-      <c r="E34" s="3"/>
+      <c r="E34" s="3">
+        <f t="shared" ref="E34:E35" si="2">G34/F34</f>
+        <v>0.46052631578947367</v>
+      </c>
       <c r="F34" s="3">
         <v>760</v>
       </c>
@@ -3697,7 +3749,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>16</v>
@@ -3706,7 +3758,10 @@
         <v>6</v>
       </c>
       <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
+      <c r="E35" s="3">
+        <f t="shared" si="2"/>
+        <v>0.62368421052631584</v>
+      </c>
       <c r="F35" s="3">
         <v>760</v>
       </c>
@@ -3747,12 +3802,12 @@
         <v>11</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>83</v>
@@ -3761,7 +3816,7 @@
         <v>10</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
@@ -3843,6 +3898,532 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:H55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="9"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="7"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
+      <c r="G30" s="7"/>
+      <c r="H30" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B39" s="6"/>
+      <c r="C39" s="6"/>
+      <c r="D39" s="6"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C42" s="3"/>
+      <c r="D42" s="3"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="B46" s="6"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B48" s="5"/>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B52" s="5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B53" s="5"/>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B54" s="5"/>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B55" s="5"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A39:D39"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{997665EB-A24E-43D9-81B6-B837BFFDEF3B}">
   <dimension ref="A1:G133"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5310,1480 +5891,6 @@
     <mergeCell ref="A50:G50"/>
     <mergeCell ref="A57:G57"/>
     <mergeCell ref="A64:G64"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G133"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="22" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B26" s="7"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="3"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="3"/>
-      <c r="G29" s="3"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
-      <c r="F30" s="3"/>
-      <c r="G30" s="3"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
-      <c r="G31" s="3"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B33" s="7"/>
-      <c r="C33" s="7"/>
-      <c r="D33" s="7"/>
-      <c r="E33" s="7"/>
-      <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
-      <c r="F35" s="3"/>
-      <c r="G35" s="3"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C36" s="3"/>
-      <c r="D36" s="3"/>
-      <c r="E36" s="3"/>
-      <c r="F36" s="3"/>
-      <c r="G36" s="3"/>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C37" s="3"/>
-      <c r="D37" s="3"/>
-      <c r="E37" s="3"/>
-      <c r="F37" s="3"/>
-      <c r="G37" s="3"/>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C38" s="3"/>
-      <c r="D38" s="3"/>
-      <c r="E38" s="3"/>
-      <c r="F38" s="3"/>
-      <c r="G38" s="3"/>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B41" s="7"/>
-      <c r="C41" s="7"/>
-      <c r="D41" s="7"/>
-      <c r="E41" s="7"/>
-      <c r="F41" s="7"/>
-      <c r="G41" s="7"/>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="B43" s="7"/>
-      <c r="C43" s="7"/>
-      <c r="D43" s="7"/>
-      <c r="E43" s="7"/>
-      <c r="F43" s="7"/>
-      <c r="G43" s="7"/>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C45" s="3"/>
-      <c r="D45" s="3"/>
-      <c r="E45" s="3"/>
-      <c r="F45" s="3"/>
-      <c r="G45" s="3"/>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C46" s="3"/>
-      <c r="D46" s="3"/>
-      <c r="E46" s="3"/>
-      <c r="F46" s="3"/>
-      <c r="G46" s="3"/>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C47" s="3"/>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
-      <c r="F47" s="3"/>
-      <c r="G47" s="3"/>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C48" s="3"/>
-      <c r="D48" s="3"/>
-      <c r="E48" s="3"/>
-      <c r="F48" s="3"/>
-      <c r="G48" s="3"/>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B50" s="7"/>
-      <c r="C50" s="7"/>
-      <c r="D50" s="7"/>
-      <c r="E50" s="7"/>
-      <c r="F50" s="7"/>
-      <c r="G50" s="7"/>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G51" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="B52" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C52" s="3"/>
-      <c r="D52" s="3"/>
-      <c r="E52" s="3"/>
-      <c r="F52" s="3"/>
-      <c r="G52" s="3"/>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C53" s="3"/>
-      <c r="D53" s="3"/>
-      <c r="E53" s="3"/>
-      <c r="F53" s="3"/>
-      <c r="G53" s="3"/>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C54" s="3"/>
-      <c r="D54" s="3"/>
-      <c r="E54" s="3"/>
-      <c r="F54" s="3"/>
-      <c r="G54" s="3"/>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C55" s="3"/>
-      <c r="D55" s="3"/>
-      <c r="E55" s="3"/>
-      <c r="F55" s="3"/>
-      <c r="G55" s="3"/>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B57" s="7"/>
-      <c r="C57" s="7"/>
-      <c r="D57" s="7"/>
-      <c r="E57" s="7"/>
-      <c r="F57" s="7"/>
-      <c r="G57" s="7"/>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F58" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G58" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A59" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="B59" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C59" s="3"/>
-      <c r="D59" s="3"/>
-      <c r="E59" s="3"/>
-      <c r="F59" s="3"/>
-      <c r="G59" s="3"/>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C60" s="3"/>
-      <c r="D60" s="3"/>
-      <c r="E60" s="3"/>
-      <c r="F60" s="3"/>
-      <c r="G60" s="3"/>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="B61" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C61" s="3"/>
-      <c r="D61" s="3"/>
-      <c r="E61" s="3"/>
-      <c r="F61" s="3"/>
-      <c r="G61" s="3"/>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C62" s="3"/>
-      <c r="D62" s="3"/>
-      <c r="E62" s="3"/>
-      <c r="F62" s="3"/>
-      <c r="G62" s="3"/>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A64" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B64" s="7"/>
-      <c r="C64" s="7"/>
-      <c r="D64" s="7"/>
-      <c r="E64" s="7"/>
-      <c r="F64" s="7"/>
-      <c r="G64" s="7"/>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A65" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E65" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F65" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G65" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C66" s="3"/>
-      <c r="D66" s="3"/>
-      <c r="E66" s="3"/>
-      <c r="F66" s="3"/>
-      <c r="G66" s="3"/>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A67" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C67" s="3"/>
-      <c r="D67" s="3"/>
-      <c r="E67" s="3"/>
-      <c r="F67" s="3"/>
-      <c r="G67" s="3"/>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C68" s="3"/>
-      <c r="D68" s="3"/>
-      <c r="E68" s="3"/>
-      <c r="F68" s="3"/>
-      <c r="G68" s="3"/>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A69" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C69" s="3"/>
-      <c r="D69" s="3"/>
-      <c r="E69" s="3"/>
-      <c r="F69" s="3"/>
-      <c r="G69" s="3"/>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B71" s="7"/>
-      <c r="C71" s="7"/>
-      <c r="D71" s="7"/>
-      <c r="E71" s="7"/>
-      <c r="F71" s="7"/>
-      <c r="G71" s="7"/>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A72" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B72" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C72" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E72" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F72" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G72" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A73" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="B73" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C73" s="3"/>
-      <c r="D73" s="3"/>
-      <c r="E73" s="3"/>
-      <c r="F73" s="3"/>
-      <c r="G73" s="3"/>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A74" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="B74" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C74" s="3"/>
-      <c r="D74" s="3"/>
-      <c r="E74" s="3"/>
-      <c r="F74" s="3"/>
-      <c r="G74" s="3"/>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A75" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="B75" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C75" s="3"/>
-      <c r="D75" s="3"/>
-      <c r="E75" s="3"/>
-      <c r="F75" s="3"/>
-      <c r="G75" s="3"/>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A76" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="B76" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C76" s="3"/>
-      <c r="D76" s="3"/>
-      <c r="E76" s="3"/>
-      <c r="F76" s="3"/>
-      <c r="G76" s="3"/>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A79" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B79" s="7"/>
-      <c r="C79" s="7"/>
-      <c r="D79" s="7"/>
-      <c r="E79" s="7"/>
-      <c r="F79" s="7"/>
-      <c r="G79" s="7"/>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A81" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="B81" s="7"/>
-      <c r="C81" s="7"/>
-      <c r="D81" s="7"/>
-      <c r="E81" s="7"/>
-      <c r="F81" s="7"/>
-      <c r="G81" s="7"/>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A82" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E82" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F82" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G82" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A83" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="B83" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C83" s="3"/>
-      <c r="D83" s="3"/>
-      <c r="E83" s="3"/>
-      <c r="F83" s="3"/>
-      <c r="G83" s="3"/>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A84" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="B84" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C84" s="3"/>
-      <c r="D84" s="3"/>
-      <c r="E84" s="3"/>
-      <c r="F84" s="3"/>
-      <c r="G84" s="3"/>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A85" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="B85" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C85" s="3"/>
-      <c r="D85" s="3"/>
-      <c r="E85" s="3"/>
-      <c r="F85" s="3"/>
-      <c r="G85" s="3"/>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A86" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="B86" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A88" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B88" s="7"/>
-      <c r="C88" s="7"/>
-      <c r="D88" s="7"/>
-      <c r="E88" s="7"/>
-      <c r="F88" s="7"/>
-      <c r="G88" s="7"/>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A89" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B89" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C89" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D89" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E89" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F89" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G89" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A90" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="B90" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C90" s="3"/>
-      <c r="D90" s="3"/>
-      <c r="E90" s="3"/>
-      <c r="F90" s="3"/>
-      <c r="G90" s="3"/>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A91" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="B91" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C91" s="3"/>
-      <c r="D91" s="3"/>
-      <c r="E91" s="3"/>
-      <c r="F91" s="3"/>
-      <c r="G91" s="3"/>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A92" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="B92" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C92" s="3"/>
-      <c r="D92" s="3"/>
-      <c r="E92" s="3"/>
-      <c r="F92" s="3"/>
-      <c r="G92" s="3"/>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A93" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="B93" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C93" s="3"/>
-      <c r="D93" s="3"/>
-      <c r="E93" s="3"/>
-      <c r="F93" s="3"/>
-      <c r="G93" s="3"/>
-    </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A95" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B95" s="7"/>
-      <c r="C95" s="7"/>
-      <c r="D95" s="7"/>
-      <c r="E95" s="7"/>
-      <c r="F95" s="7"/>
-      <c r="G95" s="7"/>
-    </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A96" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B96" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C96" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D96" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E96" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F96" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G96" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A97" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="B97" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C97" s="3"/>
-      <c r="D97" s="3"/>
-      <c r="E97" s="3"/>
-      <c r="F97" s="3"/>
-      <c r="G97" s="3"/>
-    </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A98" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="B98" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C98" s="3"/>
-      <c r="D98" s="3"/>
-      <c r="E98" s="3"/>
-      <c r="F98" s="3"/>
-      <c r="G98" s="3"/>
-    </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A99" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="B99" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C99" s="3"/>
-      <c r="D99" s="3"/>
-      <c r="E99" s="3"/>
-      <c r="F99" s="3"/>
-      <c r="G99" s="3"/>
-    </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A100" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="B100" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C100" s="3"/>
-      <c r="D100" s="3"/>
-      <c r="E100" s="3"/>
-      <c r="F100" s="3"/>
-      <c r="G100" s="3"/>
-    </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A102" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B102" s="7"/>
-      <c r="C102" s="7"/>
-      <c r="D102" s="7"/>
-      <c r="E102" s="7"/>
-      <c r="F102" s="7"/>
-      <c r="G102" s="7"/>
-    </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A103" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B103" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C103" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D103" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E103" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F103" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G103" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A104" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="B104" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C104" s="3"/>
-      <c r="D104" s="3"/>
-      <c r="E104" s="3"/>
-      <c r="F104" s="3"/>
-      <c r="G104" s="3"/>
-    </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A105" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="B105" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C105" s="3"/>
-      <c r="D105" s="3"/>
-      <c r="E105" s="3"/>
-      <c r="F105" s="3"/>
-      <c r="G105" s="3"/>
-    </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A106" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="B106" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C106" s="3"/>
-      <c r="D106" s="3"/>
-      <c r="E106" s="3"/>
-      <c r="F106" s="3"/>
-      <c r="G106" s="3"/>
-    </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A107" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="B107" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C107" s="3"/>
-      <c r="D107" s="3"/>
-      <c r="E107" s="3"/>
-      <c r="F107" s="3"/>
-      <c r="G107" s="3"/>
-    </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A109" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B109" s="7"/>
-      <c r="C109" s="7"/>
-      <c r="D109" s="7"/>
-      <c r="E109" s="7"/>
-      <c r="F109" s="7"/>
-      <c r="G109" s="7"/>
-    </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A110" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B110" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C110" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D110" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E110" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F110" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G110" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A111" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="B111" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C111" s="3"/>
-      <c r="D111" s="3"/>
-      <c r="E111" s="3"/>
-      <c r="F111" s="3"/>
-      <c r="G111" s="3"/>
-    </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A112" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="B112" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C112" s="3"/>
-      <c r="D112" s="3"/>
-      <c r="E112" s="3"/>
-      <c r="F112" s="3"/>
-      <c r="G112" s="3"/>
-    </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A113" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="B113" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C113" s="3"/>
-      <c r="D113" s="3"/>
-      <c r="E113" s="3"/>
-      <c r="F113" s="3"/>
-      <c r="G113" s="3"/>
-    </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A114" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="B114" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C114" s="3"/>
-      <c r="D114" s="3"/>
-      <c r="E114" s="3"/>
-      <c r="F114" s="3"/>
-      <c r="G114" s="3"/>
-    </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A117" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="B117" s="7"/>
-      <c r="C117" s="7"/>
-      <c r="D117" s="7"/>
-    </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A119" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B119" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C119" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="D119" s="2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A120" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="B120" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="C120" s="3"/>
-      <c r="D120" s="3"/>
-    </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A121" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="B121" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="C121" s="3"/>
-      <c r="D121" s="3"/>
-    </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A124" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="B124" s="7"/>
-    </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A126" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="B126" s="5"/>
-    </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A127" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B127" s="5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A128" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B128" s="5" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A129" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B129" s="5" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A130" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="B130" s="5" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A131" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B131" s="5"/>
-    </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A132" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="B132" s="5"/>
-    </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A133" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B133" s="5"/>
-    </row>
-  </sheetData>
-  <mergeCells count="20">
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A12:G12"/>
-    <mergeCell ref="A50:G50"/>
-    <mergeCell ref="A26:G26"/>
-    <mergeCell ref="A95:G95"/>
-    <mergeCell ref="A71:G71"/>
-    <mergeCell ref="A57:G57"/>
-    <mergeCell ref="A33:G33"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A43:G43"/>
-    <mergeCell ref="A19:G19"/>
-    <mergeCell ref="A41:G41"/>
-    <mergeCell ref="A124:B124"/>
-    <mergeCell ref="A102:G102"/>
-    <mergeCell ref="A64:G64"/>
-    <mergeCell ref="A88:G88"/>
-    <mergeCell ref="A79:G79"/>
-    <mergeCell ref="A109:G109"/>
-    <mergeCell ref="A81:G81"/>
-    <mergeCell ref="A117:D117"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>

</xml_diff>